<commit_message>
feat(templates): update and reorganize remaining aggregate test templates
</commit_message>
<xml_diff>
--- a/app/templates/informes/Informes agregado/CARAS/1-INF.-N-000-26-AG35-CARAS-ASTM-D5821-V04.xlsx
+++ b/app/templates/informes/Informes agregado/CARAS/1-INF.-N-000-26-AG35-CARAS-ASTM-D5821-V04.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Documents\crmnew\api-geofal-crm\app\templates\informes\Informes agregado\CARAS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B81EE8A-B40A-4005-AE46-740735B21F78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F06CD6BE-2E95-4CE2-BC8C-DA5843569B7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="723" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="723" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FORMATO" sheetId="1" r:id="rId1"/>
@@ -30,22 +30,22 @@
     <definedName name="_CC2">[1]Sucs!$L$6</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'caras fracturadas'!$A$1:$K$56</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">FORMATO!$B$1:$H$51</definedName>
-    <definedName name="CC" localSheetId="0">[4]Sucs!$L$6</definedName>
-    <definedName name="CC">[2]Sucs!$L$6</definedName>
-    <definedName name="CM">[3]BGA!$H$9</definedName>
-    <definedName name="CU" localSheetId="0">[4]Sucs!$L$5</definedName>
-    <definedName name="CU">[2]Sucs!$L$5</definedName>
-    <definedName name="IP" localSheetId="0">[4]Sucs!$L$4</definedName>
-    <definedName name="IP">[2]Sucs!$L$4</definedName>
-    <definedName name="Ll" localSheetId="0">[4]Sucs!$L$3</definedName>
-    <definedName name="Ll">[2]Sucs!$L$3</definedName>
-    <definedName name="MORA">[3]BGA!$H$13</definedName>
-    <definedName name="N_10" localSheetId="0">[4]Sucs!$C$5</definedName>
-    <definedName name="N_10">[2]Sucs!$C$5</definedName>
-    <definedName name="N_200" localSheetId="0">[4]Sucs!$C$3</definedName>
-    <definedName name="N_200">[2]Sucs!$C$3</definedName>
-    <definedName name="N_40" localSheetId="0">[4]Sucs!$C$4</definedName>
-    <definedName name="N_40">[2]Sucs!$C$4</definedName>
+    <definedName name="CC" localSheetId="0">[2]Sucs!$L$6</definedName>
+    <definedName name="CC">[3]Sucs!$L$6</definedName>
+    <definedName name="CM">[4]BGA!$H$9</definedName>
+    <definedName name="CU" localSheetId="0">[2]Sucs!$L$5</definedName>
+    <definedName name="CU">[3]Sucs!$L$5</definedName>
+    <definedName name="IP" localSheetId="0">[2]Sucs!$L$4</definedName>
+    <definedName name="IP">[3]Sucs!$L$4</definedName>
+    <definedName name="Ll" localSheetId="0">[2]Sucs!$L$3</definedName>
+    <definedName name="Ll">[3]Sucs!$L$3</definedName>
+    <definedName name="MORA">[4]BGA!$H$13</definedName>
+    <definedName name="N_10" localSheetId="0">[2]Sucs!$C$5</definedName>
+    <definedName name="N_10">[3]Sucs!$C$5</definedName>
+    <definedName name="N_200" localSheetId="0">[2]Sucs!$C$3</definedName>
+    <definedName name="N_200">[3]Sucs!$C$3</definedName>
+    <definedName name="N_40" localSheetId="0">[2]Sucs!$C$4</definedName>
+    <definedName name="N_40">[3]Sucs!$C$4</definedName>
     <definedName name="TABLA" localSheetId="2">#REF!</definedName>
     <definedName name="TABLA" localSheetId="0">#REF!</definedName>
     <definedName name="TABLA">#REF!</definedName>
@@ -3238,30 +3238,36 @@
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="55" xfId="0" applyBorder="1"/>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="55" xfId="0" applyBorder="1" applyProtection="1">
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="45" fillId="0" borderId="52" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="54" xfId="0" applyBorder="1" applyProtection="1">
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="45" fillId="0" borderId="52" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="54" xfId="0" applyBorder="1" applyProtection="1">
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="42" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="7" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="55" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3277,13 +3283,6 @@
     <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="3" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="45" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyProtection="1">
-      <protection hidden="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -3292,12 +3291,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="55" xfId="0" applyBorder="1" applyProtection="1">
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
@@ -3323,6 +3316,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="53" xfId="0" applyBorder="1" applyProtection="1">
       <protection hidden="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyProtection="1">
+      <protection hidden="1"/>
+    </xf>
     <xf numFmtId="173" fontId="9" fillId="2" borderId="47" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection hidden="1"/>
@@ -3337,17 +3333,30 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="41" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="42" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="45" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="5" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="5" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
@@ -3357,6 +3366,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="5" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3374,25 +3393,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
       <protection locked="0" hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="5" quotePrefix="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="5" quotePrefix="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="5" quotePrefix="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
@@ -3431,70 +3431,70 @@
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="52" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="2" fillId="2" borderId="52" xfId="4" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="1" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="166" fontId="6" fillId="2" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="15" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="2" borderId="58" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="58" xfId="0" applyBorder="1" applyProtection="1">
+    <xf numFmtId="166" fontId="6" fillId="2" borderId="13" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
     <xf numFmtId="166" fontId="6" fillId="2" borderId="15" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="177" fontId="14" fillId="0" borderId="52" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="1" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="11" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="15" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="166" fontId="6" fillId="2" borderId="10" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="52" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="2" fillId="2" borderId="52" xfId="4" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="1" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="2" borderId="13" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="14" fillId="0" borderId="52" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="1" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="2" borderId="58" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="58" xfId="0" applyBorder="1" applyProtection="1">
+      <protection hidden="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -4980,7 +4980,7 @@
       <sheetData sheetId="12" refreshError="1"/>
       <sheetData sheetId="13" refreshError="1"/>
       <sheetData sheetId="14" refreshError="1"/>
-      <sheetData sheetId="15" refreshError="1"/>
+      <sheetData sheetId="15"/>
       <sheetData sheetId="16" refreshError="1"/>
     </sheetDataSet>
   </externalBook>
@@ -4988,38 +4988,6 @@
 </file>
 
 <file path=xl/externalLinks/externalLink3.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <sheetNames>
-      <sheetName val="BGA"/>
-      <sheetName val="BGB"/>
-      <sheetName val="BGC"/>
-      <sheetName val="Hoja1"/>
-      <sheetName val="Límites"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0">
-        <row r="9">
-          <cell r="H9">
-            <v>10215</v>
-          </cell>
-        </row>
-        <row r="13">
-          <cell r="H13" t="e">
-            <v>#DIV/0!</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3"/>
-      <sheetData sheetId="4" refreshError="1"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
-</file>
-
-<file path=xl/externalLinks/externalLink4.xml><?xml version="1.0" encoding="utf-8"?>
 <externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
@@ -5087,8 +5055,40 @@
       <sheetData sheetId="12" refreshError="1"/>
       <sheetData sheetId="13" refreshError="1"/>
       <sheetData sheetId="14" refreshError="1"/>
-      <sheetData sheetId="15"/>
+      <sheetData sheetId="15" refreshError="1"/>
       <sheetData sheetId="16" refreshError="1"/>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
+</file>
+
+<file path=xl/externalLinks/externalLink4.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <sheetNames>
+      <sheetName val="BGA"/>
+      <sheetName val="BGB"/>
+      <sheetName val="BGC"/>
+      <sheetName val="Hoja1"/>
+      <sheetName val="Límites"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0">
+        <row r="9">
+          <cell r="H9">
+            <v>10215</v>
+          </cell>
+        </row>
+        <row r="13">
+          <cell r="H13" t="e">
+            <v>#DIV/0!</v>
+          </cell>
+        </row>
+      </sheetData>
+      <sheetData sheetId="1"/>
+      <sheetData sheetId="2"/>
+      <sheetData sheetId="3"/>
+      <sheetData sheetId="4" refreshError="1"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -5469,13 +5469,13 @@
     <row r="2" spans="2:11" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="341"/>
       <c r="C2" s="342"/>
-      <c r="D2" s="455" t="s">
-        <v>0</v>
-      </c>
-      <c r="E2" s="442"/>
-      <c r="F2" s="442"/>
-      <c r="G2" s="442"/>
-      <c r="H2" s="456"/>
+      <c r="D2" s="456" t="s">
+        <v>0</v>
+      </c>
+      <c r="E2" s="447"/>
+      <c r="F2" s="447"/>
+      <c r="G2" s="447"/>
+      <c r="H2" s="457"/>
       <c r="J2" s="416" t="s">
         <v>1</v>
       </c>
@@ -5484,13 +5484,13 @@
     <row r="3" spans="2:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="341"/>
       <c r="C3" s="342"/>
-      <c r="D3" s="472" t="s">
+      <c r="D3" s="470" t="s">
         <v>2</v>
       </c>
-      <c r="E3" s="473"/>
-      <c r="F3" s="473"/>
-      <c r="G3" s="473"/>
-      <c r="H3" s="474"/>
+      <c r="E3" s="471"/>
+      <c r="F3" s="471"/>
+      <c r="G3" s="471"/>
+      <c r="H3" s="472"/>
       <c r="J3" s="416" t="s">
         <v>3</v>
       </c>
@@ -5541,10 +5541,10 @@
       <c r="D7" s="350" t="s">
         <v>7</v>
       </c>
-      <c r="E7" s="476" t="s">
+      <c r="E7" s="440" t="s">
         <v>8</v>
       </c>
-      <c r="F7" s="448"/>
+      <c r="F7" s="441"/>
       <c r="G7" s="350" t="s">
         <v>9</v>
       </c>
@@ -5558,8 +5558,8 @@
       <c r="B8" s="351"/>
       <c r="C8" s="352"/>
       <c r="D8" s="352"/>
-      <c r="E8" s="447"/>
-      <c r="F8" s="448"/>
+      <c r="E8" s="449"/>
+      <c r="F8" s="441"/>
       <c r="G8" s="353"/>
       <c r="H8" s="343"/>
       <c r="J8" s="416" t="s">
@@ -5569,8 +5569,8 @@
     </row>
     <row r="9" spans="2:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="351"/>
-      <c r="C9" s="457"/>
-      <c r="D9" s="442"/>
+      <c r="C9" s="458"/>
+      <c r="D9" s="447"/>
       <c r="E9" s="354"/>
       <c r="F9" s="354"/>
       <c r="G9" s="354"/>
@@ -5592,30 +5592,30 @@
       <c r="K10" s="420"/>
     </row>
     <row r="11" spans="2:11" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="470" t="s">
+      <c r="B11" s="467" t="s">
         <v>13</v>
       </c>
-      <c r="C11" s="471"/>
-      <c r="D11" s="471"/>
-      <c r="E11" s="471"/>
-      <c r="F11" s="471"/>
-      <c r="G11" s="471"/>
-      <c r="H11" s="459"/>
+      <c r="C11" s="468"/>
+      <c r="D11" s="468"/>
+      <c r="E11" s="468"/>
+      <c r="F11" s="468"/>
+      <c r="G11" s="468"/>
+      <c r="H11" s="469"/>
       <c r="J11" s="416" t="s">
         <v>14</v>
       </c>
       <c r="K11" s="420"/>
     </row>
     <row r="12" spans="2:11" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="465" t="s">
+      <c r="B12" s="462" t="s">
         <v>15</v>
       </c>
-      <c r="C12" s="466"/>
-      <c r="D12" s="466"/>
-      <c r="E12" s="466"/>
-      <c r="F12" s="466"/>
-      <c r="G12" s="466"/>
-      <c r="H12" s="467"/>
+      <c r="C12" s="463"/>
+      <c r="D12" s="463"/>
+      <c r="E12" s="463"/>
+      <c r="F12" s="463"/>
+      <c r="G12" s="463"/>
+      <c r="H12" s="464"/>
       <c r="J12" s="416" t="s">
         <v>16</v>
       </c>
@@ -5640,18 +5640,18 @@
       <c r="C14" s="360"/>
       <c r="D14" s="361"/>
       <c r="E14" s="362"/>
-      <c r="G14" s="469" t="s">
+      <c r="G14" s="466" t="s">
         <v>19</v>
       </c>
-      <c r="H14" s="444"/>
+      <c r="H14" s="445"/>
       <c r="J14" s="419"/>
       <c r="K14" s="420"/>
     </row>
     <row r="15" spans="2:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="475" t="s">
+      <c r="B15" s="473" t="s">
         <v>20</v>
       </c>
-      <c r="C15" s="444"/>
+      <c r="C15" s="445"/>
       <c r="D15" s="290" t="s">
         <v>21</v>
       </c>
@@ -5692,8 +5692,8 @@
         <v>30</v>
       </c>
       <c r="C17" s="290"/>
-      <c r="D17" s="460"/>
-      <c r="E17" s="461"/>
+      <c r="D17" s="459"/>
+      <c r="E17" s="460"/>
       <c r="G17" s="367" t="s">
         <v>31</v>
       </c>
@@ -5716,10 +5716,10 @@
       <c r="E18" s="371" t="s">
         <v>36</v>
       </c>
-      <c r="G18" s="440" t="s">
+      <c r="G18" s="474" t="s">
         <v>37</v>
       </c>
-      <c r="H18" s="441"/>
+      <c r="H18" s="475"/>
     </row>
     <row r="19" spans="2:14" ht="16.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B19" s="372" t="s">
@@ -5729,8 +5729,8 @@
       <c r="D19" s="374"/>
       <c r="E19" s="375"/>
       <c r="F19" s="376"/>
-      <c r="G19" s="442"/>
-      <c r="H19" s="442"/>
+      <c r="G19" s="447"/>
+      <c r="H19" s="447"/>
     </row>
     <row r="20" spans="2:14" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B20" s="368" t="s">
@@ -5817,57 +5817,57 @@
       <c r="H27" s="16"/>
     </row>
     <row r="28" spans="2:14" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B28" s="479" t="s">
+      <c r="B28" s="448" t="s">
         <v>48</v>
       </c>
-      <c r="C28" s="442"/>
-      <c r="D28" s="442"/>
-      <c r="E28" s="442"/>
-      <c r="F28" s="442"/>
-      <c r="G28" s="442"/>
-      <c r="H28" s="442"/>
+      <c r="C28" s="447"/>
+      <c r="D28" s="447"/>
+      <c r="E28" s="447"/>
+      <c r="F28" s="447"/>
+      <c r="G28" s="447"/>
+      <c r="H28" s="447"/>
       <c r="L28" s="392"/>
       <c r="M28" s="392"/>
       <c r="N28" s="392"/>
     </row>
     <row r="29" spans="2:14" ht="24.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B29" s="478" t="s">
+      <c r="B29" s="446" t="s">
         <v>49</v>
       </c>
-      <c r="C29" s="442"/>
-      <c r="D29" s="442"/>
-      <c r="E29" s="442"/>
-      <c r="F29" s="442"/>
-      <c r="G29" s="442"/>
-      <c r="H29" s="442"/>
+      <c r="C29" s="447"/>
+      <c r="D29" s="447"/>
+      <c r="E29" s="447"/>
+      <c r="F29" s="447"/>
+      <c r="G29" s="447"/>
+      <c r="H29" s="447"/>
       <c r="L29" s="392"/>
       <c r="M29" s="392"/>
       <c r="N29" s="392"/>
     </row>
     <row r="30" spans="2:14" ht="16.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B30" s="445" t="s">
+      <c r="B30" s="476" t="s">
         <v>50</v>
       </c>
-      <c r="C30" s="442"/>
-      <c r="D30" s="442"/>
-      <c r="E30" s="442"/>
-      <c r="F30" s="442"/>
-      <c r="G30" s="442"/>
-      <c r="H30" s="442"/>
+      <c r="C30" s="447"/>
+      <c r="D30" s="447"/>
+      <c r="E30" s="447"/>
+      <c r="F30" s="447"/>
+      <c r="G30" s="447"/>
+      <c r="H30" s="447"/>
       <c r="L30" s="392"/>
       <c r="M30" s="392"/>
       <c r="N30" s="392"/>
     </row>
     <row r="31" spans="2:14" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B31" s="449" t="s">
+      <c r="B31" s="450" t="s">
         <v>51</v>
       </c>
-      <c r="C31" s="450"/>
-      <c r="D31" s="451"/>
-      <c r="E31" s="462" t="s">
+      <c r="C31" s="451"/>
+      <c r="D31" s="452"/>
+      <c r="E31" s="461" t="s">
         <v>52</v>
       </c>
-      <c r="F31" s="463"/>
+      <c r="F31" s="443"/>
       <c r="G31" s="393" t="s">
         <v>53</v>
       </c>
@@ -5876,13 +5876,13 @@
       <c r="N31" s="392"/>
     </row>
     <row r="32" spans="2:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B32" s="452"/>
-      <c r="C32" s="453"/>
-      <c r="D32" s="454"/>
-      <c r="E32" s="468" t="s">
+      <c r="B32" s="453"/>
+      <c r="C32" s="454"/>
+      <c r="D32" s="455"/>
+      <c r="E32" s="465" t="s">
         <v>54</v>
       </c>
-      <c r="F32" s="444"/>
+      <c r="F32" s="445"/>
       <c r="G32" s="394" t="s">
         <v>54</v>
       </c>
@@ -5899,8 +5899,8 @@
       </c>
       <c r="C33" s="396"/>
       <c r="D33" s="397"/>
-      <c r="E33" s="443"/>
-      <c r="F33" s="444"/>
+      <c r="E33" s="444"/>
+      <c r="F33" s="445"/>
       <c r="G33" s="439"/>
     </row>
     <row r="34" spans="1:8" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -5912,8 +5912,8 @@
       </c>
       <c r="C34" s="398"/>
       <c r="D34" s="377"/>
-      <c r="E34" s="443"/>
-      <c r="F34" s="444"/>
+      <c r="E34" s="444"/>
+      <c r="F34" s="445"/>
       <c r="G34" s="439"/>
     </row>
     <row r="35" spans="1:8" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -5925,18 +5925,18 @@
       </c>
       <c r="C35" s="398"/>
       <c r="D35" s="377"/>
-      <c r="E35" s="443"/>
-      <c r="F35" s="444"/>
+      <c r="E35" s="444"/>
+      <c r="F35" s="445"/>
       <c r="G35" s="244"/>
     </row>
     <row r="36" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B36" s="395"/>
       <c r="C36" s="398"/>
       <c r="D36" s="377"/>
-      <c r="E36" s="468" t="s">
+      <c r="E36" s="465" t="s">
         <v>61</v>
       </c>
-      <c r="F36" s="444"/>
+      <c r="F36" s="445"/>
       <c r="G36" s="394" t="s">
         <v>61</v>
       </c>
@@ -5947,8 +5947,8 @@
       </c>
       <c r="C37" s="398"/>
       <c r="D37" s="377"/>
-      <c r="E37" s="443"/>
-      <c r="F37" s="444"/>
+      <c r="E37" s="444"/>
+      <c r="F37" s="445"/>
       <c r="G37" s="244"/>
     </row>
     <row r="38" spans="1:8" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -5960,8 +5960,8 @@
       </c>
       <c r="C38" s="398"/>
       <c r="D38" s="377"/>
-      <c r="E38" s="443"/>
-      <c r="F38" s="444"/>
+      <c r="E38" s="444"/>
+      <c r="F38" s="445"/>
       <c r="G38" s="244"/>
     </row>
     <row r="39" spans="1:8" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -5973,8 +5973,8 @@
       </c>
       <c r="C39" s="398"/>
       <c r="D39" s="377"/>
-      <c r="E39" s="443"/>
-      <c r="F39" s="444"/>
+      <c r="E39" s="444"/>
+      <c r="F39" s="445"/>
       <c r="G39" s="244"/>
     </row>
     <row r="40" spans="1:8" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -5986,8 +5986,8 @@
       </c>
       <c r="C40" s="401"/>
       <c r="D40" s="402"/>
-      <c r="E40" s="458"/>
-      <c r="F40" s="459"/>
+      <c r="E40" s="478"/>
+      <c r="F40" s="469"/>
       <c r="G40" s="403"/>
     </row>
     <row r="41" spans="1:8" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -5996,8 +5996,8 @@
       </c>
       <c r="C41" s="398"/>
       <c r="D41" s="377"/>
-      <c r="E41" s="477"/>
-      <c r="F41" s="463"/>
+      <c r="E41" s="442"/>
+      <c r="F41" s="443"/>
       <c r="G41" s="244"/>
     </row>
     <row r="42" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -6063,24 +6063,42 @@
       <c r="B49" s="415" t="s">
         <v>68</v>
       </c>
-      <c r="E49" s="464"/>
-      <c r="F49" s="442"/>
+      <c r="E49" s="479"/>
+      <c r="F49" s="447"/>
     </row>
     <row r="50" spans="2:8" ht="7.2" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="51" spans="2:8" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B51" s="446" t="s">
+      <c r="B51" s="477" t="s">
         <v>69</v>
       </c>
-      <c r="C51" s="442"/>
-      <c r="D51" s="442"/>
-      <c r="E51" s="442"/>
-      <c r="F51" s="442"/>
-      <c r="G51" s="442"/>
-      <c r="H51" s="442"/>
+      <c r="C51" s="447"/>
+      <c r="D51" s="447"/>
+      <c r="E51" s="447"/>
+      <c r="F51" s="447"/>
+      <c r="G51" s="447"/>
+      <c r="H51" s="447"/>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="J6wxDxPGp6dUHZ4EQnGq5hntQmLWvmuKVE9IIya0ki4ZwiEtH/fJGpoRPGo33qOoPgc/p7THFufXJ69pDOPB3Q==" saltValue="FrDlFNAAFB059EZfhoU7Wg==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="28">
+    <mergeCell ref="B51:H51"/>
+    <mergeCell ref="E39:F39"/>
+    <mergeCell ref="E40:F40"/>
+    <mergeCell ref="E49:F49"/>
+    <mergeCell ref="D2:H2"/>
+    <mergeCell ref="C9:D9"/>
+    <mergeCell ref="D17:E17"/>
+    <mergeCell ref="E31:F31"/>
+    <mergeCell ref="E34:F34"/>
+    <mergeCell ref="B12:H12"/>
+    <mergeCell ref="G14:H14"/>
+    <mergeCell ref="B11:H11"/>
+    <mergeCell ref="D3:H3"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="E32:F32"/>
+    <mergeCell ref="G18:H19"/>
+    <mergeCell ref="E33:F33"/>
+    <mergeCell ref="B30:H30"/>
     <mergeCell ref="E7:F7"/>
     <mergeCell ref="E41:F41"/>
     <mergeCell ref="E37:F37"/>
@@ -6090,25 +6108,7 @@
     <mergeCell ref="E35:F35"/>
     <mergeCell ref="E38:F38"/>
     <mergeCell ref="B31:D32"/>
-    <mergeCell ref="D2:H2"/>
-    <mergeCell ref="C9:D9"/>
-    <mergeCell ref="D17:E17"/>
-    <mergeCell ref="E31:F31"/>
-    <mergeCell ref="E34:F34"/>
-    <mergeCell ref="B12:H12"/>
     <mergeCell ref="E36:F36"/>
-    <mergeCell ref="G14:H14"/>
-    <mergeCell ref="B11:H11"/>
-    <mergeCell ref="D3:H3"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="E32:F32"/>
-    <mergeCell ref="G18:H19"/>
-    <mergeCell ref="E33:F33"/>
-    <mergeCell ref="B30:H30"/>
-    <mergeCell ref="B51:H51"/>
-    <mergeCell ref="E39:F39"/>
-    <mergeCell ref="E40:F40"/>
-    <mergeCell ref="E49:F49"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0" right="0.59055118110236227" top="0.78740157480314965" bottom="0" header="0" footer="0"/>
@@ -6154,36 +6154,36 @@
       <c r="M1" s="126"/>
     </row>
     <row r="2" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="490" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="488"/>
-      <c r="C2" s="488"/>
-      <c r="D2" s="488"/>
-      <c r="E2" s="488"/>
-      <c r="F2" s="488"/>
-      <c r="G2" s="488"/>
-      <c r="H2" s="488"/>
-      <c r="I2" s="488"/>
-      <c r="J2" s="488"/>
-      <c r="K2" s="488"/>
+      <c r="A2" s="486" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="481"/>
+      <c r="C2" s="481"/>
+      <c r="D2" s="481"/>
+      <c r="E2" s="481"/>
+      <c r="F2" s="481"/>
+      <c r="G2" s="481"/>
+      <c r="H2" s="481"/>
+      <c r="I2" s="481"/>
+      <c r="J2" s="481"/>
+      <c r="K2" s="481"/>
       <c r="L2" s="128"/>
       <c r="M2" s="128"/>
     </row>
     <row r="3" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="485">
-        <v>0</v>
-      </c>
-      <c r="B3" s="486"/>
-      <c r="C3" s="486"/>
-      <c r="D3" s="486"/>
-      <c r="E3" s="486"/>
-      <c r="F3" s="486"/>
-      <c r="G3" s="486"/>
-      <c r="H3" s="486"/>
-      <c r="I3" s="486"/>
-      <c r="J3" s="486"/>
-      <c r="K3" s="486"/>
+      <c r="A3" s="491">
+        <v>0</v>
+      </c>
+      <c r="B3" s="492"/>
+      <c r="C3" s="492"/>
+      <c r="D3" s="492"/>
+      <c r="E3" s="492"/>
+      <c r="F3" s="492"/>
+      <c r="G3" s="492"/>
+      <c r="H3" s="492"/>
+      <c r="I3" s="492"/>
+      <c r="J3" s="492"/>
+      <c r="K3" s="492"/>
       <c r="L3" s="129"/>
       <c r="M3" s="129"/>
     </row>
@@ -6207,15 +6207,15 @@
       <c r="B5" s="148" t="s">
         <v>71</v>
       </c>
-      <c r="C5" s="480">
+      <c r="C5" s="483">
         <f>+FORMATO!K2</f>
         <v>0</v>
       </c>
-      <c r="D5" s="481"/>
-      <c r="E5" s="481"/>
-      <c r="F5" s="481"/>
-      <c r="G5" s="481"/>
-      <c r="H5" s="481"/>
+      <c r="D5" s="484"/>
+      <c r="E5" s="484"/>
+      <c r="F5" s="484"/>
+      <c r="G5" s="484"/>
+      <c r="H5" s="484"/>
       <c r="I5" s="7" t="s">
         <v>72</v>
       </c>
@@ -6233,15 +6233,15 @@
       <c r="B6" s="148" t="s">
         <v>71</v>
       </c>
-      <c r="C6" s="480">
+      <c r="C6" s="483">
         <f>+FORMATO!K3</f>
         <v>0</v>
       </c>
-      <c r="D6" s="481"/>
-      <c r="E6" s="481"/>
-      <c r="F6" s="481"/>
-      <c r="G6" s="481"/>
-      <c r="H6" s="481"/>
+      <c r="D6" s="484"/>
+      <c r="E6" s="484"/>
+      <c r="F6" s="484"/>
+      <c r="G6" s="484"/>
+      <c r="H6" s="484"/>
       <c r="I6" s="8" t="s">
         <v>75</v>
       </c>
@@ -6260,15 +6260,15 @@
       <c r="B7" s="148" t="s">
         <v>71</v>
       </c>
-      <c r="C7" s="480">
+      <c r="C7" s="483">
         <f>+FORMATO!K4</f>
         <v>0</v>
       </c>
-      <c r="D7" s="481"/>
-      <c r="E7" s="481"/>
-      <c r="F7" s="481"/>
-      <c r="G7" s="481"/>
-      <c r="H7" s="481"/>
+      <c r="D7" s="484"/>
+      <c r="E7" s="484"/>
+      <c r="F7" s="484"/>
+      <c r="G7" s="484"/>
+      <c r="H7" s="484"/>
       <c r="I7" s="8" t="s">
         <v>12</v>
       </c>
@@ -6288,15 +6288,15 @@
       <c r="B8" s="148" t="s">
         <v>71</v>
       </c>
-      <c r="C8" s="480">
+      <c r="C8" s="483">
         <f>+FORMATO!K5</f>
         <v>0</v>
       </c>
-      <c r="D8" s="481"/>
-      <c r="E8" s="481"/>
-      <c r="F8" s="481"/>
-      <c r="G8" s="481"/>
-      <c r="H8" s="481"/>
+      <c r="D8" s="484"/>
+      <c r="E8" s="484"/>
+      <c r="F8" s="484"/>
+      <c r="G8" s="484"/>
+      <c r="H8" s="484"/>
       <c r="I8" s="429" t="s">
         <v>78</v>
       </c>
@@ -6338,36 +6338,36 @@
       <c r="K10" s="4"/>
     </row>
     <row r="11" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="491" t="s">
+      <c r="A11" s="487" t="s">
         <v>80</v>
       </c>
-      <c r="B11" s="471"/>
-      <c r="C11" s="471"/>
-      <c r="D11" s="471"/>
-      <c r="E11" s="471"/>
-      <c r="F11" s="471"/>
-      <c r="G11" s="471"/>
-      <c r="H11" s="471"/>
-      <c r="I11" s="471"/>
-      <c r="J11" s="471"/>
-      <c r="K11" s="459"/>
+      <c r="B11" s="468"/>
+      <c r="C11" s="468"/>
+      <c r="D11" s="468"/>
+      <c r="E11" s="468"/>
+      <c r="F11" s="468"/>
+      <c r="G11" s="468"/>
+      <c r="H11" s="468"/>
+      <c r="I11" s="468"/>
+      <c r="J11" s="468"/>
+      <c r="K11" s="469"/>
       <c r="L11" s="131"/>
       <c r="M11" s="131"/>
     </row>
     <row r="12" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="483" t="s">
+      <c r="A12" s="489" t="s">
         <v>15</v>
       </c>
-      <c r="B12" s="473"/>
-      <c r="C12" s="473"/>
-      <c r="D12" s="473"/>
-      <c r="E12" s="473"/>
-      <c r="F12" s="473"/>
-      <c r="G12" s="473"/>
-      <c r="H12" s="473"/>
-      <c r="I12" s="473"/>
-      <c r="J12" s="473"/>
-      <c r="K12" s="484"/>
+      <c r="B12" s="471"/>
+      <c r="C12" s="471"/>
+      <c r="D12" s="471"/>
+      <c r="E12" s="471"/>
+      <c r="F12" s="471"/>
+      <c r="G12" s="471"/>
+      <c r="H12" s="471"/>
+      <c r="I12" s="471"/>
+      <c r="J12" s="471"/>
+      <c r="K12" s="490"/>
       <c r="L12" s="131"/>
       <c r="M12" s="136"/>
     </row>
@@ -6519,19 +6519,19 @@
       <c r="M19" s="126"/>
     </row>
     <row r="20" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="482" t="s">
+      <c r="A20" s="488" t="s">
         <v>87</v>
       </c>
-      <c r="B20" s="450"/>
-      <c r="C20" s="450"/>
-      <c r="D20" s="450"/>
-      <c r="E20" s="450"/>
-      <c r="F20" s="450"/>
-      <c r="G20" s="450"/>
-      <c r="H20" s="450"/>
-      <c r="I20" s="450"/>
-      <c r="J20" s="450"/>
-      <c r="K20" s="451"/>
+      <c r="B20" s="451"/>
+      <c r="C20" s="451"/>
+      <c r="D20" s="451"/>
+      <c r="E20" s="451"/>
+      <c r="F20" s="451"/>
+      <c r="G20" s="451"/>
+      <c r="H20" s="451"/>
+      <c r="I20" s="451"/>
+      <c r="J20" s="451"/>
+      <c r="K20" s="452"/>
       <c r="L20" s="20"/>
       <c r="M20" s="16"/>
     </row>
@@ -6600,19 +6600,19 @@
       <c r="M24" s="12"/>
     </row>
     <row r="25" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="482" t="s">
+      <c r="A25" s="488" t="s">
         <v>90</v>
       </c>
-      <c r="B25" s="450"/>
-      <c r="C25" s="450"/>
-      <c r="D25" s="450"/>
-      <c r="E25" s="450"/>
-      <c r="F25" s="450"/>
-      <c r="G25" s="450"/>
-      <c r="H25" s="450"/>
-      <c r="I25" s="450"/>
-      <c r="J25" s="450"/>
-      <c r="K25" s="451"/>
+      <c r="B25" s="451"/>
+      <c r="C25" s="451"/>
+      <c r="D25" s="451"/>
+      <c r="E25" s="451"/>
+      <c r="F25" s="451"/>
+      <c r="G25" s="451"/>
+      <c r="H25" s="451"/>
+      <c r="I25" s="451"/>
+      <c r="J25" s="451"/>
+      <c r="K25" s="452"/>
       <c r="L25" s="12"/>
       <c r="M25" s="12"/>
     </row>
@@ -6667,19 +6667,19 @@
       <c r="M28" s="12"/>
     </row>
     <row r="29" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="482" t="s">
+      <c r="A29" s="488" t="s">
         <v>92</v>
       </c>
-      <c r="B29" s="450"/>
-      <c r="C29" s="450"/>
-      <c r="D29" s="450"/>
-      <c r="E29" s="450"/>
-      <c r="F29" s="450"/>
-      <c r="G29" s="450"/>
-      <c r="H29" s="450"/>
-      <c r="I29" s="450"/>
-      <c r="J29" s="450"/>
-      <c r="K29" s="451"/>
+      <c r="B29" s="451"/>
+      <c r="C29" s="451"/>
+      <c r="D29" s="451"/>
+      <c r="E29" s="451"/>
+      <c r="F29" s="451"/>
+      <c r="G29" s="451"/>
+      <c r="H29" s="451"/>
+      <c r="I29" s="451"/>
+      <c r="J29" s="451"/>
+      <c r="K29" s="452"/>
       <c r="L29" s="12"/>
       <c r="M29" s="12"/>
     </row>
@@ -6774,19 +6774,19 @@
       <c r="M34" s="16"/>
     </row>
     <row r="35" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="482" t="s">
+      <c r="A35" s="488" t="s">
         <v>96</v>
       </c>
-      <c r="B35" s="450"/>
-      <c r="C35" s="450"/>
-      <c r="D35" s="450"/>
-      <c r="E35" s="450"/>
-      <c r="F35" s="450"/>
-      <c r="G35" s="450"/>
-      <c r="H35" s="450"/>
-      <c r="I35" s="450"/>
-      <c r="J35" s="450"/>
-      <c r="K35" s="451"/>
+      <c r="B35" s="451"/>
+      <c r="C35" s="451"/>
+      <c r="D35" s="451"/>
+      <c r="E35" s="451"/>
+      <c r="F35" s="451"/>
+      <c r="G35" s="451"/>
+      <c r="H35" s="451"/>
+      <c r="I35" s="451"/>
+      <c r="J35" s="451"/>
+      <c r="K35" s="452"/>
       <c r="L35" s="20"/>
       <c r="M35" s="16"/>
     </row>
@@ -6875,85 +6875,85 @@
       <c r="M40" s="12"/>
     </row>
     <row r="41" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="489" t="s">
+      <c r="A41" s="485" t="s">
         <v>100</v>
       </c>
-      <c r="B41" s="488"/>
-      <c r="C41" s="488"/>
-      <c r="D41" s="488"/>
-      <c r="E41" s="488"/>
-      <c r="F41" s="488"/>
-      <c r="G41" s="488"/>
-      <c r="H41" s="488"/>
-      <c r="I41" s="488"/>
-      <c r="J41" s="488"/>
-      <c r="K41" s="488"/>
+      <c r="B41" s="481"/>
+      <c r="C41" s="481"/>
+      <c r="D41" s="481"/>
+      <c r="E41" s="481"/>
+      <c r="F41" s="481"/>
+      <c r="G41" s="481"/>
+      <c r="H41" s="481"/>
+      <c r="I41" s="481"/>
+      <c r="J41" s="481"/>
+      <c r="K41" s="481"/>
       <c r="M41" s="12"/>
     </row>
     <row r="42" spans="1:14" ht="39.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="487" t="s">
+      <c r="A42" s="480" t="s">
         <v>101</v>
       </c>
-      <c r="B42" s="488"/>
-      <c r="C42" s="488"/>
-      <c r="D42" s="488"/>
-      <c r="E42" s="488"/>
-      <c r="F42" s="488"/>
-      <c r="G42" s="488"/>
-      <c r="H42" s="488"/>
-      <c r="I42" s="488"/>
-      <c r="J42" s="488"/>
-      <c r="K42" s="488"/>
+      <c r="B42" s="481"/>
+      <c r="C42" s="481"/>
+      <c r="D42" s="481"/>
+      <c r="E42" s="481"/>
+      <c r="F42" s="481"/>
+      <c r="G42" s="481"/>
+      <c r="H42" s="481"/>
+      <c r="I42" s="481"/>
+      <c r="J42" s="481"/>
+      <c r="K42" s="481"/>
       <c r="M42" s="12"/>
     </row>
     <row r="43" spans="1:14" ht="16.2" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A43" s="487" t="s">
+      <c r="A43" s="480" t="s">
         <v>102</v>
       </c>
-      <c r="B43" s="488"/>
-      <c r="C43" s="488"/>
-      <c r="D43" s="488"/>
-      <c r="E43" s="488"/>
-      <c r="F43" s="488"/>
-      <c r="G43" s="488"/>
-      <c r="H43" s="488"/>
-      <c r="I43" s="488"/>
-      <c r="J43" s="488"/>
-      <c r="K43" s="488"/>
+      <c r="B43" s="481"/>
+      <c r="C43" s="481"/>
+      <c r="D43" s="481"/>
+      <c r="E43" s="481"/>
+      <c r="F43" s="481"/>
+      <c r="G43" s="481"/>
+      <c r="H43" s="481"/>
+      <c r="I43" s="481"/>
+      <c r="J43" s="481"/>
+      <c r="K43" s="481"/>
       <c r="L43" s="134"/>
       <c r="M43" s="12"/>
     </row>
     <row r="44" spans="1:14" ht="27.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A44" s="487" t="s">
+      <c r="A44" s="480" t="s">
         <v>103</v>
       </c>
-      <c r="B44" s="488"/>
-      <c r="C44" s="488"/>
-      <c r="D44" s="488"/>
-      <c r="E44" s="488"/>
-      <c r="F44" s="488"/>
-      <c r="G44" s="488"/>
-      <c r="H44" s="488"/>
-      <c r="I44" s="488"/>
-      <c r="J44" s="488"/>
-      <c r="K44" s="488"/>
+      <c r="B44" s="481"/>
+      <c r="C44" s="481"/>
+      <c r="D44" s="481"/>
+      <c r="E44" s="481"/>
+      <c r="F44" s="481"/>
+      <c r="G44" s="481"/>
+      <c r="H44" s="481"/>
+      <c r="I44" s="481"/>
+      <c r="J44" s="481"/>
+      <c r="K44" s="481"/>
       <c r="L44" s="132"/>
       <c r="M44" s="12"/>
     </row>
     <row r="45" spans="1:14" ht="27" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A45" s="492" t="s">
+      <c r="A45" s="482" t="s">
         <v>104</v>
       </c>
-      <c r="B45" s="488"/>
-      <c r="C45" s="488"/>
-      <c r="D45" s="488"/>
-      <c r="E45" s="488"/>
-      <c r="F45" s="488"/>
-      <c r="G45" s="488"/>
-      <c r="H45" s="488"/>
-      <c r="I45" s="488"/>
-      <c r="J45" s="488"/>
-      <c r="K45" s="488"/>
+      <c r="B45" s="481"/>
+      <c r="C45" s="481"/>
+      <c r="D45" s="481"/>
+      <c r="E45" s="481"/>
+      <c r="F45" s="481"/>
+      <c r="G45" s="481"/>
+      <c r="H45" s="481"/>
+      <c r="I45" s="481"/>
+      <c r="J45" s="481"/>
+      <c r="K45" s="481"/>
       <c r="L45" s="319"/>
       <c r="M45" s="319"/>
       <c r="N45" s="319"/>
@@ -7122,11 +7122,6 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="SnhlqkvQKvkNW91AbpMF+7nJmyqqVAtsUq7pT+jTLVBrCP3lm7MjcyD0wwo4NLwXHzvLI95W9GI+JH6qIPDHQw==" saltValue="KIlZwzaYJ/wENx1fwB/IKQ==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="17">
-    <mergeCell ref="A44:K44"/>
-    <mergeCell ref="A45:K45"/>
-    <mergeCell ref="C7:H7"/>
-    <mergeCell ref="A43:K43"/>
-    <mergeCell ref="A41:K41"/>
     <mergeCell ref="A2:K2"/>
     <mergeCell ref="A11:K11"/>
     <mergeCell ref="C8:H8"/>
@@ -7139,6 +7134,11 @@
     <mergeCell ref="A29:K29"/>
     <mergeCell ref="C5:H5"/>
     <mergeCell ref="A25:K25"/>
+    <mergeCell ref="A44:K44"/>
+    <mergeCell ref="A45:K45"/>
+    <mergeCell ref="C7:H7"/>
+    <mergeCell ref="A43:K43"/>
+    <mergeCell ref="A41:K41"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" showInputMessage="1" showErrorMessage="1" sqref="K36 L35:L36" xr:uid="{00000000-0002-0000-0100-000000000000}">
@@ -7184,7 +7184,7 @@
       <c r="F1" s="502"/>
       <c r="G1" s="502"/>
       <c r="H1" s="502"/>
-      <c r="I1" s="463"/>
+      <c r="I1" s="443"/>
     </row>
     <row r="2" spans="1:14" ht="4.2" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="3" spans="1:14" ht="12" customHeight="1" x14ac:dyDescent="0.25">
@@ -7193,7 +7193,7 @@
       </c>
       <c r="C3" s="502"/>
       <c r="D3" s="502"/>
-      <c r="E3" s="463"/>
+      <c r="E3" s="443"/>
       <c r="F3" s="184"/>
       <c r="G3" s="249" t="s">
         <v>110</v>
@@ -7623,9 +7623,9 @@
     </row>
     <row r="24" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B24" s="496"/>
-      <c r="C24" s="466"/>
-      <c r="D24" s="466"/>
-      <c r="E24" s="467"/>
+      <c r="C24" s="463"/>
+      <c r="D24" s="463"/>
+      <c r="E24" s="464"/>
       <c r="F24" s="207" t="s">
         <v>143</v>
       </c>
@@ -8022,16 +8022,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="525"/>
-      <c r="B1" s="451"/>
-      <c r="C1" s="520" t="s">
+      <c r="A1" s="517"/>
+      <c r="B1" s="452"/>
+      <c r="C1" s="508" t="s">
         <v>150</v>
       </c>
-      <c r="D1" s="450"/>
-      <c r="E1" s="450"/>
-      <c r="F1" s="450"/>
-      <c r="G1" s="450"/>
-      <c r="H1" s="451"/>
+      <c r="D1" s="451"/>
+      <c r="E1" s="451"/>
+      <c r="F1" s="451"/>
+      <c r="G1" s="451"/>
+      <c r="H1" s="452"/>
       <c r="I1" s="22" t="s">
         <v>151</v>
       </c>
@@ -8040,14 +8040,14 @@
       </c>
     </row>
     <row r="2" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="521"/>
-      <c r="B2" s="513"/>
-      <c r="C2" s="521"/>
-      <c r="D2" s="511"/>
-      <c r="E2" s="511"/>
-      <c r="F2" s="511"/>
-      <c r="G2" s="511"/>
-      <c r="H2" s="513"/>
+      <c r="A2" s="509"/>
+      <c r="B2" s="511"/>
+      <c r="C2" s="509"/>
+      <c r="D2" s="510"/>
+      <c r="E2" s="510"/>
+      <c r="F2" s="510"/>
+      <c r="G2" s="510"/>
+      <c r="H2" s="511"/>
       <c r="I2" s="22" t="s">
         <v>153</v>
       </c>
@@ -8056,14 +8056,14 @@
       </c>
     </row>
     <row r="3" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="521"/>
-      <c r="B3" s="513"/>
-      <c r="C3" s="521"/>
-      <c r="D3" s="511"/>
-      <c r="E3" s="511"/>
-      <c r="F3" s="511"/>
-      <c r="G3" s="511"/>
-      <c r="H3" s="513"/>
+      <c r="A3" s="509"/>
+      <c r="B3" s="511"/>
+      <c r="C3" s="509"/>
+      <c r="D3" s="510"/>
+      <c r="E3" s="510"/>
+      <c r="F3" s="510"/>
+      <c r="G3" s="510"/>
+      <c r="H3" s="511"/>
       <c r="I3" s="22" t="s">
         <v>154</v>
       </c>
@@ -8072,14 +8072,14 @@
       </c>
     </row>
     <row r="4" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="452"/>
-      <c r="B4" s="454"/>
-      <c r="C4" s="452"/>
-      <c r="D4" s="453"/>
-      <c r="E4" s="453"/>
-      <c r="F4" s="453"/>
-      <c r="G4" s="453"/>
-      <c r="H4" s="454"/>
+      <c r="A4" s="453"/>
+      <c r="B4" s="455"/>
+      <c r="C4" s="453"/>
+      <c r="D4" s="454"/>
+      <c r="E4" s="454"/>
+      <c r="F4" s="454"/>
+      <c r="G4" s="454"/>
+      <c r="H4" s="455"/>
       <c r="I4" s="22" t="s">
         <v>155</v>
       </c>
@@ -8091,17 +8091,17 @@
       <c r="A6" s="25" t="s">
         <v>157</v>
       </c>
-      <c r="B6" s="516" t="s">
+      <c r="B6" s="504" t="s">
         <v>80</v>
       </c>
-      <c r="C6" s="517"/>
-      <c r="D6" s="517"/>
-      <c r="E6" s="517"/>
-      <c r="F6" s="517"/>
-      <c r="G6" s="517"/>
-      <c r="H6" s="517"/>
-      <c r="I6" s="517"/>
-      <c r="J6" s="461"/>
+      <c r="C6" s="505"/>
+      <c r="D6" s="505"/>
+      <c r="E6" s="505"/>
+      <c r="F6" s="505"/>
+      <c r="G6" s="505"/>
+      <c r="H6" s="505"/>
+      <c r="I6" s="505"/>
+      <c r="J6" s="460"/>
     </row>
     <row r="7" spans="1:10" ht="16.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="25" t="s">
@@ -8381,10 +8381,10 @@
         <v>182</v>
       </c>
       <c r="I26" s="50"/>
-      <c r="J26" s="518" t="s">
+      <c r="J26" s="506" t="s">
         <v>183</v>
       </c>
-      <c r="K26" s="448"/>
+      <c r="K26" s="441"/>
       <c r="L26" s="284" t="s">
         <v>184</v>
       </c>
@@ -8435,11 +8435,11 @@
       <c r="I27" s="303" t="s">
         <v>136</v>
       </c>
-      <c r="J27" s="515" t="str">
+      <c r="J27" s="522" t="str">
         <f>+A27</f>
         <v xml:space="preserve">Masa de la muestra &gt; 3/8 (g), </v>
       </c>
-      <c r="K27" s="459"/>
+      <c r="K27" s="469"/>
       <c r="L27" s="282">
         <f>+H27</f>
         <v>0</v>
@@ -8488,11 +8488,11 @@
         <v>182</v>
       </c>
       <c r="I28" s="50"/>
-      <c r="J28" s="509" t="str">
+      <c r="J28" s="515" t="str">
         <f>+A31</f>
         <v xml:space="preserve">Masa de la muestra &lt; 3/8 (g), </v>
       </c>
-      <c r="K28" s="484"/>
+      <c r="K28" s="490"/>
       <c r="L28" s="283">
         <f>+H31</f>
         <v>0</v>
@@ -8541,11 +8541,11 @@
         <v>182</v>
       </c>
       <c r="I29" s="50"/>
-      <c r="J29" s="505" t="str">
+      <c r="J29" s="520" t="str">
         <f>+A36</f>
         <v>Masa particulas Fracturadas (g)</v>
       </c>
-      <c r="K29" s="484"/>
+      <c r="K29" s="490"/>
       <c r="L29" s="283" t="e">
         <f>+H36</f>
         <v>#DIV/0!</v>
@@ -8594,11 +8594,11 @@
         <v>182</v>
       </c>
       <c r="I30" s="50"/>
-      <c r="J30" s="512" t="str">
+      <c r="J30" s="518" t="str">
         <f>+A40</f>
         <v>Masa particulas que no cumplen el criterio especificado (g)</v>
       </c>
-      <c r="K30" s="513"/>
+      <c r="K30" s="511"/>
       <c r="L30" s="283" t="e">
         <f>+H40</f>
         <v>#DIV/0!</v>
@@ -8651,11 +8651,11 @@
       <c r="I31" s="303" t="s">
         <v>138</v>
       </c>
-      <c r="J31" s="509" t="str">
+      <c r="J31" s="515" t="str">
         <f>+A45</f>
         <v>Masa particulas Fracturadas (g)</v>
       </c>
-      <c r="K31" s="484"/>
+      <c r="K31" s="490"/>
       <c r="L31" s="283">
         <f>+H45</f>
         <v>0</v>
@@ -8704,11 +8704,11 @@
         <v>182</v>
       </c>
       <c r="I32" s="50"/>
-      <c r="J32" s="504" t="str">
+      <c r="J32" s="513" t="str">
         <f>+A49</f>
         <v>Masa particulas que no cumplen el criterio especificado (g)</v>
       </c>
-      <c r="K32" s="484"/>
+      <c r="K32" s="490"/>
       <c r="L32" s="283">
         <f>+H49</f>
         <v>0</v>
@@ -8757,11 +8757,11 @@
         <v>182</v>
       </c>
       <c r="I33" s="50"/>
-      <c r="J33" s="514" t="str">
+      <c r="J33" s="519" t="str">
         <f>+A53</f>
         <v xml:space="preserve">factor de presición </v>
       </c>
-      <c r="K33" s="467"/>
+      <c r="K33" s="464"/>
       <c r="L33" s="283">
         <f>+H53</f>
         <v>0.5837</v>
@@ -9789,10 +9789,10 @@
         <v>182</v>
       </c>
       <c r="I58" s="50"/>
-      <c r="J58" s="518" t="s">
+      <c r="J58" s="506" t="s">
         <v>183</v>
       </c>
-      <c r="K58" s="448"/>
+      <c r="K58" s="441"/>
       <c r="L58" s="284" t="s">
         <v>184</v>
       </c>
@@ -9841,11 +9841,11 @@
       <c r="I59" s="303" t="s">
         <v>136</v>
       </c>
-      <c r="J59" s="507" t="str">
+      <c r="J59" s="524" t="str">
         <f>+A59</f>
         <v xml:space="preserve">Masa de la muestra &gt; 3/8 (g), </v>
       </c>
-      <c r="K59" s="508"/>
+      <c r="K59" s="525"/>
       <c r="L59" s="282">
         <f>+H59</f>
         <v>0</v>
@@ -9892,11 +9892,11 @@
         <v>182</v>
       </c>
       <c r="I60" s="50"/>
-      <c r="J60" s="509" t="str">
+      <c r="J60" s="515" t="str">
         <f>+A63</f>
         <v xml:space="preserve">Masa de la muestra &lt; 3/8 (g), </v>
       </c>
-      <c r="K60" s="484"/>
+      <c r="K60" s="490"/>
       <c r="L60" s="283">
         <f>+H63</f>
         <v>0</v>
@@ -9943,11 +9943,11 @@
         <v>182</v>
       </c>
       <c r="I61" s="50"/>
-      <c r="J61" s="505" t="str">
+      <c r="J61" s="520" t="str">
         <f>+A68</f>
         <v>Masa particulas Fracturadas (g)</v>
       </c>
-      <c r="K61" s="484"/>
+      <c r="K61" s="490"/>
       <c r="L61" s="283" t="e">
         <f>+H68</f>
         <v>#DIV/0!</v>
@@ -9996,11 +9996,11 @@
         <v>182</v>
       </c>
       <c r="I62" s="50"/>
-      <c r="J62" s="512" t="str">
+      <c r="J62" s="518" t="str">
         <f>+A72</f>
         <v>Masa particulas que no cumplen el criterio especificado (g)</v>
       </c>
-      <c r="K62" s="513"/>
+      <c r="K62" s="511"/>
       <c r="L62" s="283" t="e">
         <f>+H72</f>
         <v>#DIV/0!</v>
@@ -10053,11 +10053,11 @@
       <c r="I63" s="303" t="s">
         <v>138</v>
       </c>
-      <c r="J63" s="523" t="str">
+      <c r="J63" s="514" t="str">
         <f>+A77</f>
         <v>Masa particulas Fracturadas (g)</v>
       </c>
-      <c r="K63" s="484"/>
+      <c r="K63" s="490"/>
       <c r="L63" s="283">
         <f>+H77</f>
         <v>0</v>
@@ -10093,11 +10093,11 @@
         <v>182</v>
       </c>
       <c r="I64" s="50"/>
-      <c r="J64" s="504" t="str">
+      <c r="J64" s="513" t="str">
         <f>+A81</f>
         <v>Masa particulas que no cumplen el criterio especificado (g)</v>
       </c>
-      <c r="K64" s="484"/>
+      <c r="K64" s="490"/>
       <c r="L64" s="283">
         <f>+H81</f>
         <v>0</v>
@@ -10133,11 +10133,11 @@
         <v>182</v>
       </c>
       <c r="I65" s="50"/>
-      <c r="J65" s="514" t="str">
+      <c r="J65" s="519" t="str">
         <f>+A85</f>
         <v xml:space="preserve">factor de presición </v>
       </c>
-      <c r="K65" s="467"/>
+      <c r="K65" s="464"/>
       <c r="L65" s="283">
         <f>+H85</f>
         <v>0.65808729579660641</v>
@@ -10808,19 +10808,19 @@
       <c r="A90" s="431" t="s">
         <v>198</v>
       </c>
-      <c r="B90" s="506" t="s">
+      <c r="B90" s="523" t="s">
         <v>199</v>
       </c>
-      <c r="C90" s="461"/>
+      <c r="C90" s="460"/>
       <c r="D90" s="432"/>
-      <c r="E90" s="522" t="s">
+      <c r="E90" s="512" t="s">
         <v>200</v>
       </c>
-      <c r="F90" s="511"/>
-      <c r="G90" s="524" t="s">
+      <c r="F90" s="510"/>
+      <c r="G90" s="516" t="s">
         <v>201</v>
       </c>
-      <c r="H90" s="461"/>
+      <c r="H90" s="460"/>
     </row>
     <row r="91" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A91" s="32"/>
@@ -10836,23 +10836,32 @@
       <c r="A92" s="433" t="s">
         <v>202</v>
       </c>
-      <c r="B92" s="519">
+      <c r="B92" s="507">
         <v>45604</v>
       </c>
-      <c r="C92" s="461"/>
+      <c r="C92" s="460"/>
       <c r="D92" s="32"/>
-      <c r="E92" s="510" t="s">
+      <c r="E92" s="521" t="s">
         <v>203</v>
       </c>
-      <c r="F92" s="511"/>
-      <c r="G92" s="519">
+      <c r="F92" s="510"/>
+      <c r="G92" s="507">
         <v>45605</v>
       </c>
-      <c r="H92" s="461"/>
+      <c r="H92" s="460"/>
     </row>
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="8bpvulMySDhbCinMJCKA6z/Rt8I37vsDQJVa4PyGNTLespzr8fQA8IH94JgjrRjZWt4j2jiXTM/mppn7uL1Pfg==" saltValue="zH87836e9WKbmOJcNpq46A==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="25">
+    <mergeCell ref="B90:C90"/>
+    <mergeCell ref="J59:K59"/>
+    <mergeCell ref="J28:K28"/>
+    <mergeCell ref="J60:K60"/>
+    <mergeCell ref="J30:K30"/>
+    <mergeCell ref="J65:K65"/>
+    <mergeCell ref="J27:K27"/>
+    <mergeCell ref="J64:K64"/>
+    <mergeCell ref="J29:K29"/>
     <mergeCell ref="B6:J6"/>
     <mergeCell ref="J26:K26"/>
     <mergeCell ref="G92:H92"/>
@@ -10869,15 +10878,6 @@
     <mergeCell ref="J61:K61"/>
     <mergeCell ref="J58:K58"/>
     <mergeCell ref="E92:F92"/>
-    <mergeCell ref="J60:K60"/>
-    <mergeCell ref="J30:K30"/>
-    <mergeCell ref="J65:K65"/>
-    <mergeCell ref="J27:K27"/>
-    <mergeCell ref="J64:K64"/>
-    <mergeCell ref="J29:K29"/>
-    <mergeCell ref="B90:C90"/>
-    <mergeCell ref="J59:K59"/>
-    <mergeCell ref="J28:K28"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>
@@ -11382,8 +11382,8 @@
       <c r="B7" s="530">
         <v>0.5837</v>
       </c>
-      <c r="C7" s="517"/>
-      <c r="D7" s="448"/>
+      <c r="C7" s="505"/>
+      <c r="D7" s="441"/>
       <c r="E7" s="435"/>
       <c r="G7" s="123" t="s">
         <v>220</v>
@@ -11391,8 +11391,8 @@
       <c r="H7" s="532">
         <v>0.65808729579660641</v>
       </c>
-      <c r="I7" s="517"/>
-      <c r="J7" s="461"/>
+      <c r="I7" s="505"/>
+      <c r="J7" s="460"/>
     </row>
     <row r="8" spans="1:10" ht="23.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="123" t="s">
@@ -11401,8 +11401,8 @@
       <c r="B8" s="531">
         <v>0.61960000000000004</v>
       </c>
-      <c r="C8" s="517"/>
-      <c r="D8" s="448"/>
+      <c r="C8" s="505"/>
+      <c r="D8" s="441"/>
       <c r="E8" s="435"/>
       <c r="G8" s="123" t="s">
         <v>221</v>
@@ -11410,8 +11410,8 @@
       <c r="H8" s="529">
         <v>0.6933088938022407</v>
       </c>
-      <c r="I8" s="517"/>
-      <c r="J8" s="461"/>
+      <c r="I8" s="505"/>
+      <c r="J8" s="460"/>
     </row>
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="UdVjHZ9s4rk2Q1BahGxKD/MhsXkoE+GSNvJHwherni5/TVyUiNOf2Y6PcpIRg4QNJKUmMAyuGnsSMeGhc9g1aw==" saltValue="t7E+Do148jGMo7EsFdaxQg==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>

</xml_diff>